<commit_message>
Set up renv, freeze, and GitHub Pages workflow
</commit_message>
<xml_diff>
--- a/posts/2024-11-04_openxlsx/Sales_Report_2023.xlsx
+++ b/posts/2024-11-04_openxlsx/Sales_Report_2023.xlsx
@@ -62,8 +62,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="4">
@@ -140,7 +139,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>

</xml_diff>